<commit_message>
Add completed SOV answer-key and download UI
Expose a gated answer-key download for the Schedule-of-Values exercise and generate a completed workbook.

- UI: ExerciseComponent now shows a downloadable answerKey card after submission, uses NEXT_PUBLIC_BASE_PATH for public asset path, and adds the Download icon.
- Types: Added AnswerKeyDownload and answerKey field on Exercise.
- Data: activity-data populated the exercise with answerKey metadata pointing to /downloads/sov-32m-project-completed.xlsx.
- Files: added public/downloads/sov-32m-project-completed.xlsx and updated the existing sov-32m-project.xlsx.
- Script: generate-sov-workbook.py now accepts a completed flag, generates both blank and completed workbooks, and fills in formulas, SUMIFS subtotals, project totals, and formatting for the completed workbook.

Purpose: provide trainees a completed reference workbook (revealed only after they submit) so they can compare their formulas and totals against the answer key.
</commit_message>
<xml_diff>
--- a/public/downloads/sov-32m-project.xlsx
+++ b/public/downloads/sov-32m-project.xlsx
@@ -135,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,8 +152,9 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -161,14 +162,28 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -660,11 +675,11 @@
       <c r="F6" s="7" t="n">
         <v>150000</v>
       </c>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
       <c r="L6" s="5" t="n"/>
     </row>
     <row r="7">
@@ -690,11 +705,11 @@
       <c r="F7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
       <c r="L7" s="5" t="n"/>
     </row>
     <row r="8">
@@ -720,11 +735,11 @@
       <c r="F8" s="7" t="n">
         <v>44000</v>
       </c>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
       <c r="L8" s="5" t="n"/>
     </row>
     <row r="9">
@@ -750,11 +765,11 @@
       <c r="F9" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
       <c r="L9" s="5" t="n"/>
     </row>
     <row r="10">
@@ -780,11 +795,11 @@
       <c r="F10" s="7" t="n">
         <v>21000</v>
       </c>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
       <c r="L10" s="5" t="n"/>
     </row>
     <row r="11">
@@ -810,11 +825,11 @@
       <c r="F11" s="7" t="n">
         <v>210000</v>
       </c>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="8" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
       <c r="L11" s="5" t="n"/>
     </row>
     <row r="12">
@@ -840,11 +855,11 @@
       <c r="F12" s="7" t="n">
         <v>70000</v>
       </c>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
       <c r="L12" s="5" t="n"/>
     </row>
     <row r="13">
@@ -870,11 +885,11 @@
       <c r="F13" s="7" t="n">
         <v>180000</v>
       </c>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
       <c r="L13" s="5" t="n"/>
     </row>
     <row r="14">
@@ -900,11 +915,11 @@
       <c r="F14" s="7" t="n">
         <v>93600</v>
       </c>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
       <c r="L14" s="5" t="n"/>
     </row>
     <row r="15">
@@ -930,11 +945,11 @@
       <c r="F15" s="7" t="n">
         <v>101600</v>
       </c>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8" t="n"/>
-      <c r="K15" s="8" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
       <c r="L15" s="5" t="n"/>
     </row>
     <row r="16">
@@ -960,11 +975,11 @@
       <c r="F16" s="7" t="n">
         <v>330000</v>
       </c>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="8" t="n"/>
-      <c r="J16" s="8" t="n"/>
-      <c r="K16" s="8" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
       <c r="L16" s="5" t="n"/>
     </row>
     <row r="17">
@@ -990,11 +1005,11 @@
       <c r="F17" s="7" t="n">
         <v>88000</v>
       </c>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="9" t="n"/>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8" t="n"/>
-      <c r="K17" s="8" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
       <c r="L17" s="5" t="n"/>
     </row>
     <row r="18">
@@ -1020,11 +1035,11 @@
       <c r="F18" s="7" t="n">
         <v>22400</v>
       </c>
-      <c r="G18" s="8" t="n"/>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8" t="n"/>
-      <c r="K18" s="8" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
       <c r="L18" s="5" t="n"/>
     </row>
     <row r="19">
@@ -1050,11 +1065,11 @@
       <c r="F19" s="7" t="n">
         <v>318000</v>
       </c>
-      <c r="G19" s="8" t="n"/>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="n"/>
-      <c r="K19" s="8" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
       <c r="L19" s="5" t="n"/>
     </row>
     <row r="20">
@@ -1080,11 +1095,11 @@
       <c r="F20" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="8" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="8" t="n"/>
-      <c r="J20" s="8" t="n"/>
-      <c r="K20" s="8" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
       <c r="L20" s="5" t="n"/>
     </row>
     <row r="21">
@@ -1110,11 +1125,11 @@
       <c r="F21" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="8" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
       <c r="L21" s="5" t="n"/>
     </row>
     <row r="22">
@@ -1140,11 +1155,11 @@
       <c r="F22" s="7" t="n">
         <v>296000</v>
       </c>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="8" t="n"/>
-      <c r="J22" s="8" t="n"/>
-      <c r="K22" s="8" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
       <c r="L22" s="5" t="n"/>
     </row>
     <row r="23">
@@ -1170,11 +1185,11 @@
       <c r="F23" s="7" t="n">
         <v>160000</v>
       </c>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8" t="n"/>
-      <c r="K23" s="8" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
       <c r="L23" s="5" t="n"/>
     </row>
     <row r="24">
@@ -1200,11 +1215,11 @@
       <c r="F24" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="8" t="n"/>
-      <c r="H24" s="9" t="n"/>
-      <c r="I24" s="8" t="n"/>
-      <c r="J24" s="8" t="n"/>
-      <c r="K24" s="8" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
       <c r="L24" s="5" t="n"/>
     </row>
     <row r="25">
@@ -1230,11 +1245,11 @@
       <c r="F25" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="9" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="8" t="n"/>
-      <c r="K25" s="8" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
       <c r="L25" s="5" t="n"/>
     </row>
     <row r="26">
@@ -1260,174 +1275,174 @@
       <c r="F26" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="9" t="n"/>
-      <c r="I26" s="8" t="n"/>
-      <c r="J26" s="8" t="n"/>
-      <c r="K26" s="8" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="n"/>
+      <c r="K26" s="7" t="n"/>
       <c r="L26" s="5" t="n"/>
     </row>
     <row r="27" ht="8" customHeight="1"/>
     <row r="28">
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>DIVISION SUBTOTALS</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>01 — General Requirements</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="13" t="n"/>
-      <c r="H29" s="14" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="11" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="14" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>02 — Existing Conditions</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="14" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="13" t="n"/>
-      <c r="K30" s="13" t="n"/>
-      <c r="L30" s="11" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>03 — Concrete</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n"/>
-      <c r="G31" s="13" t="n"/>
-      <c r="H31" s="14" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="11" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="14" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>05 — Metals</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="14" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="13" t="n"/>
-      <c r="L32" s="11" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>31 — Earthwork</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="14" t="n"/>
-      <c r="I33" s="13" t="n"/>
-      <c r="J33" s="13" t="n"/>
-      <c r="K33" s="13" t="n"/>
-      <c r="L33" s="11" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="12" t="n"/>
+      <c r="J33" s="12" t="n"/>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="14" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>33 — Utilities</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="14" t="n"/>
-      <c r="I34" s="13" t="n"/>
-      <c r="J34" s="13" t="n"/>
-      <c r="K34" s="13" t="n"/>
-      <c r="L34" s="11" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="12" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="14" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>35 — Marine Construction</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>(SUMIFS by division — formula needed)</t>
         </is>
       </c>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="13" t="n"/>
-      <c r="H35" s="14" t="n"/>
-      <c r="I35" s="13" t="n"/>
-      <c r="J35" s="13" t="n"/>
-      <c r="K35" s="13" t="n"/>
-      <c r="L35" s="11" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="12" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="14" t="n"/>
     </row>
     <row r="36" ht="8" customHeight="1"/>
     <row r="37">
@@ -1450,66 +1465,66 @@
       <c r="I37" s="17" t="n"/>
       <c r="J37" s="17" t="n"/>
       <c r="K37" s="17" t="n"/>
-      <c r="L37" s="15" t="n"/>
+      <c r="L37" s="19" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="19" t="inlineStr">
+      <c r="B40" s="20" t="inlineStr">
         <is>
           <t>Notes for the formula columns:</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Total Billed (G)         =  Previously Billed (E) + This Period (F)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>% Complete (H)           =  Total Billed (G) / Total Contract Amount (D)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t>Remaining (I)            =  Total Contract Amount (D) − Total Billed (G)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>Retention 10% (J)        =  Total Billed (G) × 10%</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>Net Earned to Date (K)   =  Total Billed (G) − Retention (J)</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="21" t="inlineStr">
         <is>
           <t>Status (L)               =  COMPLETE | NEAR COMPLETE (≥90%) | IN PROGRESS (&gt;0%) | NOT STARTED (0%)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B47" s="21" t="inlineStr">
         <is>
           <t>Division subtotals       =  SUMIFS by division (one row per division)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="B48" s="20" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>Project Total            =  SUM of each numeric column across all line items</t>
         </is>

</xml_diff>